<commit_message>
minor bug fixes and improvements
</commit_message>
<xml_diff>
--- a/data/templates/TemPlates.xlsx
+++ b/data/templates/TemPlates.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28619"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://csiroau-my.sharepoint.com/personal/loa012_csiro_au/Documents/Python Scripts/uv_pyeast/data/templates/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\loa012\Python\PYEAST\data\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="56" documentId="8_{D9448E71-7E0A-4E00-B5F4-1F1CFBC485B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7776CE2A-1DF3-4019-8A85-773FAE209C0C}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3838260E-59CB-444E-87CD-5CBFD4C8625E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21220" firstSheet="1" activeTab="1" xr2:uid="{A88A2E90-7DAA-42AF-87DB-C66679F60F68}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" firstSheet="1" activeTab="1" xr2:uid="{A88A2E90-7DAA-42AF-87DB-C66679F60F68}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
   <si>
     <t xml:space="preserve">This is a database of templates useful for assembly of plasmids. </t>
   </si>
@@ -63,15 +63,9 @@
     <t>pVio_AmVHPO</t>
   </si>
   <si>
-    <t>pTwHC_AlphaHbGSHA_Sc</t>
-  </si>
-  <si>
     <t>B</t>
   </si>
   <si>
-    <t>pU3d_PmM_PmN</t>
-  </si>
-  <si>
     <t>mCherry-pTwistAmp-Highcopy</t>
   </si>
   <si>
@@ -90,9 +84,6 @@
     <t>pUC19-POT1KO-His</t>
   </si>
   <si>
-    <t>pLIRhide3</t>
-  </si>
-  <si>
     <t>D</t>
   </si>
   <si>
@@ -102,9 +93,6 @@
     <t>pYES2</t>
   </si>
   <si>
-    <t>pR-hp-3-ns</t>
-  </si>
-  <si>
     <t>pTw_Leu2MX_from_pRG205M</t>
   </si>
   <si>
@@ -114,12 +102,6 @@
     <t>pUC19-yEMRFP</t>
   </si>
   <si>
-    <t>pTwHC_Bt_CrtI_Sc</t>
-  </si>
-  <si>
-    <t>pR-hp-3</t>
-  </si>
-  <si>
     <t>pRS-AmVHPO-ePTS1</t>
   </si>
   <si>
@@ -129,35 +111,23 @@
     <t>s288c</t>
   </si>
   <si>
-    <t>pTwHc_Pa_CrtB_Sc</t>
-  </si>
-  <si>
-    <t>pGal1-HH-1-His3</t>
-  </si>
-  <si>
     <t>G</t>
   </si>
   <si>
     <t>YeGFP-pTwistAmp-Highcopy</t>
   </si>
   <si>
-    <t>pTwHC_Pa_CrtE_Sc</t>
-  </si>
-  <si>
     <t>H</t>
   </si>
   <si>
     <t>pVio_Ura3_2u</t>
-  </si>
-  <si>
-    <t>pTsHCamp-SIR-LIR</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -523,24 +493,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B4F0098-CC36-4333-AF7A-F1E4AB09078D}">
   <dimension ref="A1:A5"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:1">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:1">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -553,17 +523,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{037BC273-E296-4EA5-990F-78F8FA846E03}">
   <dimension ref="A1:M10"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="7" max="7" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:13">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
       <c r="B2">
         <v>1</v>
       </c>
@@ -601,7 +571,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:13">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -611,109 +581,79 @@
       <c r="C3" t="s">
         <v>7</v>
       </c>
-      <c r="D3" t="s">
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="4" spans="1:13">
-      <c r="A4" t="s">
+      <c r="C4" t="s">
         <v>9</v>
       </c>
-      <c r="B4" t="s">
+      <c r="D4" t="s">
         <v>10</v>
       </c>
-      <c r="C4" t="s">
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
         <v>11</v>
       </c>
-      <c r="D4" t="s">
+      <c r="B5" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="5" spans="1:13">
-      <c r="A5" t="s">
+      <c r="C5" t="s">
         <v>13</v>
       </c>
-      <c r="B5" t="s">
+      <c r="D5" t="s">
         <v>14</v>
       </c>
-      <c r="C5" t="s">
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
         <v>15</v>
       </c>
-      <c r="D5" t="s">
+      <c r="B6" t="s">
         <v>16</v>
       </c>
-      <c r="E5" t="s">
+      <c r="C6" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="6" spans="1:13">
-      <c r="A6" t="s">
+      <c r="E6" t="s">
         <v>18</v>
       </c>
-      <c r="B6" t="s">
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
         <v>19</v>
       </c>
-      <c r="C6" t="s">
+      <c r="B7" t="s">
         <v>20</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E7" t="s">
         <v>21</v>
       </c>
-      <c r="E6" t="s">
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7" t="s">
+      <c r="B8" t="s">
         <v>23</v>
       </c>
-      <c r="B7" t="s">
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
         <v>24</v>
       </c>
-      <c r="C7" t="s">
+      <c r="B9" t="s">
         <v>25</v>
       </c>
-      <c r="D7" t="s">
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
         <v>26</v>
       </c>
-      <c r="E7" t="s">
+      <c r="B10" t="s">
         <v>27</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13">
-      <c r="A8" t="s">
-        <v>28</v>
-      </c>
-      <c r="B8" t="s">
-        <v>29</v>
-      </c>
-      <c r="C8" t="s">
-        <v>30</v>
-      </c>
-      <c r="D8" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13">
-      <c r="A9" t="s">
-        <v>32</v>
-      </c>
-      <c r="B9" t="s">
-        <v>33</v>
-      </c>
-      <c r="C9" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13">
-      <c r="A10" t="s">
-        <v>35</v>
-      </c>
-      <c r="B10" t="s">
-        <v>36</v>
-      </c>
-      <c r="C10" t="s">
-        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
combinatorial sequence selection added to gg_lvl1. Run with with gglvl1 command
</commit_message>
<xml_diff>
--- a/data/templates/TemPlates.xlsx
+++ b/data/templates/TemPlates.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\loa012\Python\PYEAST\data\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\u5390772\Desktop\Code\PYEAST Local\data\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3838260E-59CB-444E-87CD-5CBFD4C8625E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FF4E50E-4C1F-428D-A455-AA29E71A0F27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" firstSheet="1" activeTab="1" xr2:uid="{A88A2E90-7DAA-42AF-87DB-C66679F60F68}"/>
+    <workbookView xWindow="-28920" yWindow="-975" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{A88A2E90-7DAA-42AF-87DB-C66679F60F68}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
   <si>
     <t xml:space="preserve">This is a database of templates useful for assembly of plasmids. </t>
   </si>
@@ -121,6 +121,9 @@
   </si>
   <si>
     <t>pVio_Ura3_2u</t>
+  </si>
+  <si>
+    <t>pTw_His3MX</t>
   </si>
 </sst>
 </file>
@@ -493,24 +496,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B4F0098-CC36-4333-AF7A-F1E4AB09078D}">
   <dimension ref="A1:A5"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -523,17 +526,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{037BC273-E296-4EA5-990F-78F8FA846E03}">
   <dimension ref="A1:M10"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="7" max="7" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B2">
         <v>1</v>
       </c>
@@ -571,7 +574,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -582,7 +585,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -593,7 +596,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>11</v>
       </c>
@@ -607,7 +610,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>15</v>
       </c>
@@ -621,7 +624,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>19</v>
       </c>
@@ -632,15 +635,18 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>22</v>
       </c>
       <c r="B8" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="E8" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>24</v>
       </c>
@@ -648,7 +654,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>26</v>
       </c>

</xml_diff>

<commit_message>
First working version of ggytklvl1 added. Lots of jank to be fixed before pushing to main.
</commit_message>
<xml_diff>
--- a/data/templates/TemPlates.xlsx
+++ b/data/templates/TemPlates.xlsx
@@ -8,13 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\u5390772\Desktop\Code\PYEAST Local\data\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FF4E50E-4C1F-428D-A455-AA29E71A0F27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08BFC403-4809-4EAB-BE0B-9FA86CA65CC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-975" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{A88A2E90-7DAA-42AF-87DB-C66679F60F68}"/>
+    <workbookView xWindow="-165" yWindow="-165" windowWidth="16530" windowHeight="28410" firstSheet="1" activeTab="2" xr2:uid="{A88A2E90-7DAA-42AF-87DB-C66679F60F68}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
     <sheet name="TemPlate 1" sheetId="2" r:id="rId2"/>
+    <sheet name="YTK MoClo" sheetId="3" r:id="rId3"/>
+    <sheet name="YSD MoClo" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -37,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="161">
   <si>
     <t xml:space="preserve">This is a database of templates useful for assembly of plasmids. </t>
   </si>
@@ -124,19 +126,427 @@
   </si>
   <si>
     <t>pTw_His3MX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YTK MoClo - Addgene </t>
+  </si>
+  <si>
+    <t>YSD - MoClo Addgene</t>
+  </si>
+  <si>
+    <t>pYTK001</t>
+  </si>
+  <si>
+    <t>pYTK002</t>
+  </si>
+  <si>
+    <t>pYTK003</t>
+  </si>
+  <si>
+    <t>pYTK004</t>
+  </si>
+  <si>
+    <t>pYTK005</t>
+  </si>
+  <si>
+    <t>pYTK006</t>
+  </si>
+  <si>
+    <t>pYTK007</t>
+  </si>
+  <si>
+    <t>pYTK008</t>
+  </si>
+  <si>
+    <t>pYTK009</t>
+  </si>
+  <si>
+    <t>pYTK010</t>
+  </si>
+  <si>
+    <t>pYTK011</t>
+  </si>
+  <si>
+    <t>pYTK012</t>
+  </si>
+  <si>
+    <t>pYTK013</t>
+  </si>
+  <si>
+    <t>pYTK014</t>
+  </si>
+  <si>
+    <t>pYTK015</t>
+  </si>
+  <si>
+    <t>pYTK016</t>
+  </si>
+  <si>
+    <t>pYTK017</t>
+  </si>
+  <si>
+    <t>pYTK018</t>
+  </si>
+  <si>
+    <t>pYTK019</t>
+  </si>
+  <si>
+    <t>pYTK020</t>
+  </si>
+  <si>
+    <t>pYTK021</t>
+  </si>
+  <si>
+    <t>pYTK022</t>
+  </si>
+  <si>
+    <t>pYTK023</t>
+  </si>
+  <si>
+    <t>pYTK024</t>
+  </si>
+  <si>
+    <t>pYTK025</t>
+  </si>
+  <si>
+    <t>pYTK026</t>
+  </si>
+  <si>
+    <t>pYTK027</t>
+  </si>
+  <si>
+    <t>pYTK028</t>
+  </si>
+  <si>
+    <t>pYTK029</t>
+  </si>
+  <si>
+    <t>pYTK030</t>
+  </si>
+  <si>
+    <t>pYTK031</t>
+  </si>
+  <si>
+    <t>pYTK032</t>
+  </si>
+  <si>
+    <t>pYTK033</t>
+  </si>
+  <si>
+    <t>pYTK034</t>
+  </si>
+  <si>
+    <t>pYTK035</t>
+  </si>
+  <si>
+    <t>pYTK036</t>
+  </si>
+  <si>
+    <t>pYTK037</t>
+  </si>
+  <si>
+    <t>pYTK038</t>
+  </si>
+  <si>
+    <t>pYTK039</t>
+  </si>
+  <si>
+    <t>pYTK040</t>
+  </si>
+  <si>
+    <t>pYTK041</t>
+  </si>
+  <si>
+    <t>pYTK042</t>
+  </si>
+  <si>
+    <t>pYTK043</t>
+  </si>
+  <si>
+    <t>pYTK044</t>
+  </si>
+  <si>
+    <t>pYTK045</t>
+  </si>
+  <si>
+    <t>pYTK046</t>
+  </si>
+  <si>
+    <t>pYTK047</t>
+  </si>
+  <si>
+    <t>pYTK048</t>
+  </si>
+  <si>
+    <t>pYTK049</t>
+  </si>
+  <si>
+    <t>pYTK050</t>
+  </si>
+  <si>
+    <t>pYTK051</t>
+  </si>
+  <si>
+    <t>pYTK052</t>
+  </si>
+  <si>
+    <t>pYTK053</t>
+  </si>
+  <si>
+    <t>pYTK054</t>
+  </si>
+  <si>
+    <t>pYTK055</t>
+  </si>
+  <si>
+    <t>pYTK056</t>
+  </si>
+  <si>
+    <t>pYTK057</t>
+  </si>
+  <si>
+    <t>pYTK058</t>
+  </si>
+  <si>
+    <t>pYTK059</t>
+  </si>
+  <si>
+    <t>pYTK060</t>
+  </si>
+  <si>
+    <t>pYTK061</t>
+  </si>
+  <si>
+    <t>pYTK062</t>
+  </si>
+  <si>
+    <t>pYTK063</t>
+  </si>
+  <si>
+    <t>pYTK064</t>
+  </si>
+  <si>
+    <t>pYTK065</t>
+  </si>
+  <si>
+    <t>pYTK066</t>
+  </si>
+  <si>
+    <t>pYTK067</t>
+  </si>
+  <si>
+    <t>pYTK068</t>
+  </si>
+  <si>
+    <t>pYTK069</t>
+  </si>
+  <si>
+    <t>pYTK070</t>
+  </si>
+  <si>
+    <t>pYTK071</t>
+  </si>
+  <si>
+    <t>pYTK072</t>
+  </si>
+  <si>
+    <t>pYTK073</t>
+  </si>
+  <si>
+    <t>pYTK074</t>
+  </si>
+  <si>
+    <t>pYTK075</t>
+  </si>
+  <si>
+    <t>pYTK076</t>
+  </si>
+  <si>
+    <t>pYTK077</t>
+  </si>
+  <si>
+    <t>pYTK078</t>
+  </si>
+  <si>
+    <t>pYTK079</t>
+  </si>
+  <si>
+    <t>pYTK080</t>
+  </si>
+  <si>
+    <t>pYTK081</t>
+  </si>
+  <si>
+    <t>pYTK082</t>
+  </si>
+  <si>
+    <t>pYTK083</t>
+  </si>
+  <si>
+    <t>pYTK084</t>
+  </si>
+  <si>
+    <t>pYTK085</t>
+  </si>
+  <si>
+    <t>pYTK086</t>
+  </si>
+  <si>
+    <t>pYTK087</t>
+  </si>
+  <si>
+    <t>pYTK088</t>
+  </si>
+  <si>
+    <t>pYTK089</t>
+  </si>
+  <si>
+    <t>pYTK090</t>
+  </si>
+  <si>
+    <t>pYTK091</t>
+  </si>
+  <si>
+    <t>pYTK092</t>
+  </si>
+  <si>
+    <t>pYTK093</t>
+  </si>
+  <si>
+    <t>pYTK094</t>
+  </si>
+  <si>
+    <t>pYTK095</t>
+  </si>
+  <si>
+    <t>pYTK096</t>
+  </si>
+  <si>
+    <t>pYSD001</t>
+  </si>
+  <si>
+    <t>pYSD002</t>
+  </si>
+  <si>
+    <t>pYSD003</t>
+  </si>
+  <si>
+    <t>pYSD004</t>
+  </si>
+  <si>
+    <t>pYSD005</t>
+  </si>
+  <si>
+    <t>pYSD006</t>
+  </si>
+  <si>
+    <t>pYSD007</t>
+  </si>
+  <si>
+    <t>pYSD008</t>
+  </si>
+  <si>
+    <t>pYSD009</t>
+  </si>
+  <si>
+    <t>pYSD021</t>
+  </si>
+  <si>
+    <t>pYSD022</t>
+  </si>
+  <si>
+    <t>pYSD023</t>
+  </si>
+  <si>
+    <t>pYSD024</t>
+  </si>
+  <si>
+    <t>pYSD041</t>
+  </si>
+  <si>
+    <t>pYSD042</t>
+  </si>
+  <si>
+    <t>pYSD043</t>
+  </si>
+  <si>
+    <t>pYSD044</t>
+  </si>
+  <si>
+    <t>pYSD061</t>
+  </si>
+  <si>
+    <t>pYSD063</t>
+  </si>
+  <si>
+    <t>pYSD080</t>
+  </si>
+  <si>
+    <t>pYSD081</t>
+  </si>
+  <si>
+    <t>pYSD082</t>
+  </si>
+  <si>
+    <t>pYSD083</t>
+  </si>
+  <si>
+    <t>pYSD084</t>
+  </si>
+  <si>
+    <t>pYSD085</t>
+  </si>
+  <si>
+    <t>pYSD099</t>
+  </si>
+  <si>
+    <t>pYSD100</t>
+  </si>
+  <si>
+    <t>pYSD101</t>
+  </si>
+  <si>
+    <t>pYSD113</t>
+  </si>
+  <si>
+    <t>pYSD140</t>
+  </si>
+  <si>
+    <t>pYSD141</t>
+  </si>
+  <si>
+    <t>pYSD153</t>
+  </si>
+  <si>
+    <t>pYSD300</t>
+  </si>
+  <si>
+    <t>pYSD313</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="2">
@@ -156,14 +566,28 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{EDE5F87D-B3EA-4650-9C3B-D41237AC891C}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -665,4 +1089,784 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B7AF15B-BE0C-4662-844E-430129F87998}">
+  <dimension ref="A1:M10"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>2</v>
+      </c>
+      <c r="D2">
+        <v>3</v>
+      </c>
+      <c r="E2">
+        <v>4</v>
+      </c>
+      <c r="F2">
+        <v>5</v>
+      </c>
+      <c r="G2">
+        <v>6</v>
+      </c>
+      <c r="H2">
+        <v>7</v>
+      </c>
+      <c r="I2">
+        <v>8</v>
+      </c>
+      <c r="J2">
+        <v>9</v>
+      </c>
+      <c r="K2">
+        <v>10</v>
+      </c>
+      <c r="L2">
+        <v>11</v>
+      </c>
+      <c r="M2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="M3" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="M4" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="L5" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="M5" s="3" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="J6" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="K6" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="L6" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="M6" s="4" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="J7" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="K7" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="L7" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="M7" s="4" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="I8" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="J8" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="K8" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="L8" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="M8" s="4" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>24</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="I9" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="J9" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="K9" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="L9" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="M9" s="4" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>26</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="I10" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="J10" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="K10" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="L10" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="M10" s="4" t="s">
+        <v>126</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8007E387-4B4E-4288-9FC9-B528CD4F9483}">
+  <dimension ref="A1:M72"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>2</v>
+      </c>
+      <c r="D2">
+        <v>3</v>
+      </c>
+      <c r="E2">
+        <v>4</v>
+      </c>
+      <c r="F2">
+        <v>5</v>
+      </c>
+      <c r="G2">
+        <v>6</v>
+      </c>
+      <c r="H2">
+        <v>7</v>
+      </c>
+      <c r="I2">
+        <v>8</v>
+      </c>
+      <c r="J2">
+        <v>9</v>
+      </c>
+      <c r="K2">
+        <v>10</v>
+      </c>
+      <c r="L2">
+        <v>11</v>
+      </c>
+      <c r="M2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" t="s">
+        <v>127</v>
+      </c>
+      <c r="C3" t="s">
+        <v>128</v>
+      </c>
+      <c r="D3" t="s">
+        <v>129</v>
+      </c>
+      <c r="E3" t="s">
+        <v>130</v>
+      </c>
+      <c r="F3" t="s">
+        <v>131</v>
+      </c>
+      <c r="G3" t="s">
+        <v>132</v>
+      </c>
+      <c r="H3" t="s">
+        <v>133</v>
+      </c>
+      <c r="I3" t="s">
+        <v>134</v>
+      </c>
+      <c r="J3" t="s">
+        <v>135</v>
+      </c>
+      <c r="K3" t="s">
+        <v>136</v>
+      </c>
+      <c r="L3" t="s">
+        <v>137</v>
+      </c>
+      <c r="M3" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" t="s">
+        <v>139</v>
+      </c>
+      <c r="C4" t="s">
+        <v>140</v>
+      </c>
+      <c r="D4" t="s">
+        <v>141</v>
+      </c>
+      <c r="E4" t="s">
+        <v>142</v>
+      </c>
+      <c r="F4" t="s">
+        <v>143</v>
+      </c>
+      <c r="G4" t="s">
+        <v>144</v>
+      </c>
+      <c r="H4" t="s">
+        <v>145</v>
+      </c>
+      <c r="I4" t="s">
+        <v>146</v>
+      </c>
+      <c r="J4" t="s">
+        <v>147</v>
+      </c>
+      <c r="K4" t="s">
+        <v>148</v>
+      </c>
+      <c r="L4" t="s">
+        <v>149</v>
+      </c>
+      <c r="M4" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" t="s">
+        <v>151</v>
+      </c>
+      <c r="C5" t="s">
+        <v>152</v>
+      </c>
+      <c r="D5" t="s">
+        <v>153</v>
+      </c>
+      <c r="E5" t="s">
+        <v>154</v>
+      </c>
+      <c r="F5" t="s">
+        <v>155</v>
+      </c>
+      <c r="G5" t="s">
+        <v>156</v>
+      </c>
+      <c r="H5" t="s">
+        <v>157</v>
+      </c>
+      <c r="I5" t="s">
+        <v>158</v>
+      </c>
+      <c r="J5" t="s">
+        <v>159</v>
+      </c>
+      <c r="K5" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="C13" s="4"/>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="C14" s="4"/>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="C15" s="4"/>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="C16" s="4"/>
+    </row>
+    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C17" s="4"/>
+    </row>
+    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C18" s="4"/>
+    </row>
+    <row r="19" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C19" s="4"/>
+    </row>
+    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C20" s="4"/>
+    </row>
+    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B21" s="2"/>
+      <c r="C21" s="4"/>
+      <c r="F21" s="1"/>
+    </row>
+    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B22" s="2"/>
+      <c r="C22" s="4"/>
+      <c r="F22" s="1"/>
+    </row>
+    <row r="23" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B23" s="2"/>
+      <c r="C23" s="4"/>
+      <c r="F23" s="1"/>
+    </row>
+    <row r="24" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B24" s="2"/>
+      <c r="C24" s="4"/>
+      <c r="F24" s="1"/>
+    </row>
+    <row r="25" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B25" s="2"/>
+      <c r="C25" s="4"/>
+      <c r="F25" s="1"/>
+    </row>
+    <row r="26" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B26" s="2"/>
+      <c r="C26" s="4"/>
+      <c r="F26" s="1"/>
+    </row>
+    <row r="27" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B27" s="2"/>
+      <c r="C27" s="4"/>
+      <c r="F27" s="1"/>
+    </row>
+    <row r="28" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B28" s="2"/>
+      <c r="C28" s="4"/>
+      <c r="F28" s="1"/>
+    </row>
+    <row r="29" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B29" s="2"/>
+      <c r="C29" s="4"/>
+      <c r="F29" s="1"/>
+    </row>
+    <row r="30" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B30" s="2"/>
+      <c r="C30" s="4"/>
+      <c r="F30" s="1"/>
+    </row>
+    <row r="31" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B31" s="2"/>
+      <c r="C31" s="4"/>
+      <c r="F31" s="1"/>
+    </row>
+    <row r="32" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B32" s="2"/>
+      <c r="C32" s="4"/>
+      <c r="F32" s="1"/>
+    </row>
+    <row r="33" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C33" s="4"/>
+    </row>
+    <row r="34" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C34" s="4"/>
+    </row>
+    <row r="35" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C35" s="4"/>
+    </row>
+    <row r="36" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C36" s="4"/>
+    </row>
+    <row r="37" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C37" s="4"/>
+    </row>
+    <row r="38" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C38" s="4"/>
+    </row>
+    <row r="39" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C39" s="4"/>
+    </row>
+    <row r="40" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C40" s="4"/>
+    </row>
+    <row r="41" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C41" s="4"/>
+    </row>
+    <row r="42" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C42" s="4"/>
+    </row>
+    <row r="43" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C43" s="4"/>
+    </row>
+    <row r="44" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C44" s="4"/>
+    </row>
+    <row r="45" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C45" s="4"/>
+    </row>
+    <row r="46" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C46" s="4"/>
+    </row>
+    <row r="47" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C47" s="4"/>
+    </row>
+    <row r="48" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C48" s="4"/>
+    </row>
+    <row r="49" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C49" s="4"/>
+    </row>
+    <row r="50" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C50" s="4"/>
+    </row>
+    <row r="51" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C51" s="4"/>
+    </row>
+    <row r="52" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C52" s="4"/>
+    </row>
+    <row r="53" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C53" s="4"/>
+    </row>
+    <row r="54" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C54" s="4"/>
+    </row>
+    <row r="55" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C55" s="4"/>
+    </row>
+    <row r="56" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C56" s="4"/>
+    </row>
+    <row r="57" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C57" s="4"/>
+    </row>
+    <row r="58" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C58" s="4"/>
+    </row>
+    <row r="59" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C59" s="4"/>
+    </row>
+    <row r="60" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C60" s="4"/>
+    </row>
+    <row r="61" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C61" s="4"/>
+    </row>
+    <row r="62" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C62" s="4"/>
+    </row>
+    <row r="63" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C63" s="4"/>
+    </row>
+    <row r="64" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C64" s="4"/>
+    </row>
+    <row r="65" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C65" s="4"/>
+    </row>
+    <row r="66" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C66" s="4"/>
+    </row>
+    <row r="67" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C67" s="4"/>
+    </row>
+    <row r="68" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C68" s="4"/>
+    </row>
+    <row r="69" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C69" s="4"/>
+    </row>
+    <row r="70" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C70" s="4"/>
+    </row>
+    <row r="71" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C71" s="4"/>
+    </row>
+    <row r="72" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C72" s="4"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Simplified some of the worklist outputs
</commit_message>
<xml_diff>
--- a/data/templates/TemPlates.xlsx
+++ b/data/templates/TemPlates.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\u5390772\Desktop\Code\PYEAST Local\data\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08BFC403-4809-4EAB-BE0B-9FA86CA65CC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E01AF9DF-25D8-4262-A9F6-901CDB027C87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-165" yWindow="-165" windowWidth="16530" windowHeight="28410" firstSheet="1" activeTab="2" xr2:uid="{A88A2E90-7DAA-42AF-87DB-C66679F60F68}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="16440" windowHeight="28320" firstSheet="1" activeTab="3" xr2:uid="{A88A2E90-7DAA-42AF-87DB-C66679F60F68}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="162">
   <si>
     <t xml:space="preserve">This is a database of templates useful for assembly of plasmids. </t>
   </si>
@@ -522,6 +522,9 @@
   </si>
   <si>
     <t>pYSD313</t>
+  </si>
+  <si>
+    <t>SiTag_in_pTwist_Chlor</t>
   </si>
 </sst>
 </file>
@@ -570,17 +573,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1143,40 +1137,40 @@
       <c r="A3" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="G3" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="H3" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="I3" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="J3" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="K3" s="2" t="s">
+      <c r="K3" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="L3" s="2" t="s">
+      <c r="L3" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="M3" s="2" t="s">
+      <c r="M3" s="1" t="s">
         <v>42</v>
       </c>
     </row>
@@ -1184,40 +1178,40 @@
       <c r="A4" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="F4" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="G4" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="H4" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="I4" s="2" t="s">
+      <c r="I4" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="J4" s="2" t="s">
+      <c r="J4" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="K4" s="2" t="s">
+      <c r="K4" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="L4" s="2" t="s">
+      <c r="L4" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="M4" s="2" t="s">
+      <c r="M4" s="1" t="s">
         <v>54</v>
       </c>
     </row>
@@ -1225,40 +1219,40 @@
       <c r="A5" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F5" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="G5" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="H5" s="3" t="s">
+      <c r="H5" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="I5" s="3" t="s">
+      <c r="I5" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="J5" s="3" t="s">
+      <c r="J5" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="K5" s="3" t="s">
+      <c r="K5" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="L5" s="3" t="s">
+      <c r="L5" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="M5" s="3" t="s">
+      <c r="M5" s="1" t="s">
         <v>66</v>
       </c>
     </row>
@@ -1266,40 +1260,40 @@
       <c r="A6" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E6" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="F6" s="4" t="s">
+      <c r="F6" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="G6" s="4" t="s">
+      <c r="G6" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="H6" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="I6" s="4" t="s">
+      <c r="I6" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="J6" s="4" t="s">
+      <c r="J6" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="K6" s="4" t="s">
+      <c r="K6" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="L6" s="4" t="s">
+      <c r="L6" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="M6" s="4" t="s">
+      <c r="M6" s="1" t="s">
         <v>78</v>
       </c>
     </row>
@@ -1307,40 +1301,40 @@
       <c r="A7" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E7" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="F7" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="G7" s="4" t="s">
+      <c r="G7" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="H7" s="4" t="s">
+      <c r="H7" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="I7" s="4" t="s">
+      <c r="I7" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="J7" s="4" t="s">
+      <c r="J7" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="K7" s="4" t="s">
+      <c r="K7" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="L7" s="4" t="s">
+      <c r="L7" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="M7" s="4" t="s">
+      <c r="M7" s="1" t="s">
         <v>90</v>
       </c>
     </row>
@@ -1348,40 +1342,40 @@
       <c r="A8" t="s">
         <v>22</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D8" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="E8" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="F8" s="4" t="s">
+      <c r="F8" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="G8" s="4" t="s">
+      <c r="G8" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="H8" s="4" t="s">
+      <c r="H8" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="I8" s="4" t="s">
+      <c r="I8" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="J8" s="4" t="s">
+      <c r="J8" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="K8" s="4" t="s">
+      <c r="K8" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="L8" s="4" t="s">
+      <c r="L8" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="M8" s="4" t="s">
+      <c r="M8" s="1" t="s">
         <v>102</v>
       </c>
     </row>
@@ -1389,40 +1383,40 @@
       <c r="A9" t="s">
         <v>24</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D9" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="E9" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="F9" s="4" t="s">
+      <c r="F9" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="G9" s="4" t="s">
+      <c r="G9" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="H9" s="4" t="s">
+      <c r="H9" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="I9" s="4" t="s">
+      <c r="I9" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="J9" s="4" t="s">
+      <c r="J9" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="K9" s="4" t="s">
+      <c r="K9" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="L9" s="4" t="s">
+      <c r="L9" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="M9" s="4" t="s">
+      <c r="M9" s="1" t="s">
         <v>114</v>
       </c>
     </row>
@@ -1430,40 +1424,40 @@
       <c r="A10" t="s">
         <v>26</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="D10" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="E10" s="4" t="s">
+      <c r="E10" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F10" s="4" t="s">
+      <c r="F10" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G10" s="4" t="s">
+      <c r="G10" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="H10" s="4" t="s">
+      <c r="H10" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="I10" s="4" t="s">
+      <c r="I10" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="J10" s="4" t="s">
+      <c r="J10" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="K10" s="4" t="s">
+      <c r="K10" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="L10" s="4" t="s">
+      <c r="L10" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="M10" s="4" t="s">
+      <c r="M10" s="1" t="s">
         <v>126</v>
       </c>
     </row>
@@ -1661,210 +1655,213 @@
       <c r="A10" t="s">
         <v>26</v>
       </c>
+      <c r="B10" t="s">
+        <v>161</v>
+      </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="C13" s="4"/>
+      <c r="C13" s="1"/>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="C14" s="4"/>
+      <c r="C14" s="1"/>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="C15" s="4"/>
+      <c r="C15" s="1"/>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="C16" s="4"/>
+      <c r="C16" s="1"/>
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="C17" s="4"/>
+      <c r="C17" s="1"/>
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="C18" s="4"/>
+      <c r="C18" s="1"/>
     </row>
     <row r="19" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="C19" s="4"/>
+      <c r="C19" s="1"/>
     </row>
     <row r="20" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="C20" s="4"/>
+      <c r="C20" s="1"/>
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B21" s="2"/>
-      <c r="C21" s="4"/>
+      <c r="B21" s="1"/>
+      <c r="C21" s="1"/>
       <c r="F21" s="1"/>
     </row>
     <row r="22" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B22" s="2"/>
-      <c r="C22" s="4"/>
+      <c r="B22" s="1"/>
+      <c r="C22" s="1"/>
       <c r="F22" s="1"/>
     </row>
     <row r="23" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B23" s="2"/>
-      <c r="C23" s="4"/>
+      <c r="B23" s="1"/>
+      <c r="C23" s="1"/>
       <c r="F23" s="1"/>
     </row>
     <row r="24" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B24" s="2"/>
-      <c r="C24" s="4"/>
+      <c r="B24" s="1"/>
+      <c r="C24" s="1"/>
       <c r="F24" s="1"/>
     </row>
     <row r="25" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B25" s="2"/>
-      <c r="C25" s="4"/>
+      <c r="B25" s="1"/>
+      <c r="C25" s="1"/>
       <c r="F25" s="1"/>
     </row>
     <row r="26" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B26" s="2"/>
-      <c r="C26" s="4"/>
+      <c r="B26" s="1"/>
+      <c r="C26" s="1"/>
       <c r="F26" s="1"/>
     </row>
     <row r="27" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B27" s="2"/>
-      <c r="C27" s="4"/>
+      <c r="B27" s="1"/>
+      <c r="C27" s="1"/>
       <c r="F27" s="1"/>
     </row>
     <row r="28" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B28" s="2"/>
-      <c r="C28" s="4"/>
+      <c r="B28" s="1"/>
+      <c r="C28" s="1"/>
       <c r="F28" s="1"/>
     </row>
     <row r="29" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B29" s="2"/>
-      <c r="C29" s="4"/>
+      <c r="B29" s="1"/>
+      <c r="C29" s="1"/>
       <c r="F29" s="1"/>
     </row>
     <row r="30" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B30" s="2"/>
-      <c r="C30" s="4"/>
+      <c r="B30" s="1"/>
+      <c r="C30" s="1"/>
       <c r="F30" s="1"/>
     </row>
     <row r="31" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B31" s="2"/>
-      <c r="C31" s="4"/>
+      <c r="B31" s="1"/>
+      <c r="C31" s="1"/>
       <c r="F31" s="1"/>
     </row>
     <row r="32" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B32" s="2"/>
-      <c r="C32" s="4"/>
+      <c r="B32" s="1"/>
+      <c r="C32" s="1"/>
       <c r="F32" s="1"/>
     </row>
     <row r="33" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C33" s="4"/>
+      <c r="C33" s="1"/>
     </row>
     <row r="34" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C34" s="4"/>
+      <c r="C34" s="1"/>
     </row>
     <row r="35" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C35" s="4"/>
+      <c r="C35" s="1"/>
     </row>
     <row r="36" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C36" s="4"/>
+      <c r="C36" s="1"/>
     </row>
     <row r="37" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C37" s="4"/>
+      <c r="C37" s="1"/>
     </row>
     <row r="38" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C38" s="4"/>
+      <c r="C38" s="1"/>
     </row>
     <row r="39" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C39" s="4"/>
+      <c r="C39" s="1"/>
     </row>
     <row r="40" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C40" s="4"/>
+      <c r="C40" s="1"/>
     </row>
     <row r="41" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C41" s="4"/>
+      <c r="C41" s="1"/>
     </row>
     <row r="42" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C42" s="4"/>
+      <c r="C42" s="1"/>
     </row>
     <row r="43" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C43" s="4"/>
+      <c r="C43" s="1"/>
     </row>
     <row r="44" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C44" s="4"/>
+      <c r="C44" s="1"/>
     </row>
     <row r="45" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C45" s="4"/>
+      <c r="C45" s="1"/>
     </row>
     <row r="46" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C46" s="4"/>
+      <c r="C46" s="1"/>
     </row>
     <row r="47" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C47" s="4"/>
+      <c r="C47" s="1"/>
     </row>
     <row r="48" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C48" s="4"/>
+      <c r="C48" s="1"/>
     </row>
     <row r="49" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C49" s="4"/>
+      <c r="C49" s="1"/>
     </row>
     <row r="50" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C50" s="4"/>
+      <c r="C50" s="1"/>
     </row>
     <row r="51" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C51" s="4"/>
+      <c r="C51" s="1"/>
     </row>
     <row r="52" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C52" s="4"/>
+      <c r="C52" s="1"/>
     </row>
     <row r="53" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C53" s="4"/>
+      <c r="C53" s="1"/>
     </row>
     <row r="54" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C54" s="4"/>
+      <c r="C54" s="1"/>
     </row>
     <row r="55" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C55" s="4"/>
+      <c r="C55" s="1"/>
     </row>
     <row r="56" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C56" s="4"/>
+      <c r="C56" s="1"/>
     </row>
     <row r="57" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C57" s="4"/>
+      <c r="C57" s="1"/>
     </row>
     <row r="58" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C58" s="4"/>
+      <c r="C58" s="1"/>
     </row>
     <row r="59" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C59" s="4"/>
+      <c r="C59" s="1"/>
     </row>
     <row r="60" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C60" s="4"/>
+      <c r="C60" s="1"/>
     </row>
     <row r="61" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C61" s="4"/>
+      <c r="C61" s="1"/>
     </row>
     <row r="62" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C62" s="4"/>
+      <c r="C62" s="1"/>
     </row>
     <row r="63" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C63" s="4"/>
+      <c r="C63" s="1"/>
     </row>
     <row r="64" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C64" s="4"/>
+      <c r="C64" s="1"/>
     </row>
     <row r="65" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C65" s="4"/>
+      <c r="C65" s="1"/>
     </row>
     <row r="66" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C66" s="4"/>
+      <c r="C66" s="1"/>
     </row>
     <row r="67" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C67" s="4"/>
+      <c r="C67" s="1"/>
     </row>
     <row r="68" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C68" s="4"/>
+      <c r="C68" s="1"/>
     </row>
     <row r="69" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C69" s="4"/>
+      <c r="C69" s="1"/>
     </row>
     <row r="70" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C70" s="4"/>
+      <c r="C70" s="1"/>
     </row>
     <row r="71" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C71" s="4"/>
+      <c r="C71" s="1"/>
     </row>
     <row r="72" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C72" s="4"/>
+      <c r="C72" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
GG feature almost finished now Support added for Yeast MoClo and OpenPichia
</commit_message>
<xml_diff>
--- a/data/templates/TemPlates.xlsx
+++ b/data/templates/TemPlates.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\u5390772\Desktop\Code\PYEAST Local\data\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E01AF9DF-25D8-4262-A9F6-901CDB027C87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D22DF228-8826-4673-9617-DF0650F21D70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="16440" windowHeight="28320" firstSheet="1" activeTab="3" xr2:uid="{A88A2E90-7DAA-42AF-87DB-C66679F60F68}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="16440" windowHeight="28320" firstSheet="1" activeTab="4" xr2:uid="{A88A2E90-7DAA-42AF-87DB-C66679F60F68}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
     <sheet name="TemPlate 1" sheetId="2" r:id="rId2"/>
     <sheet name="YTK MoClo" sheetId="3" r:id="rId3"/>
     <sheet name="YSD MoClo" sheetId="4" r:id="rId4"/>
+    <sheet name="Open Pichia" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="223">
   <si>
     <t xml:space="preserve">This is a database of templates useful for assembly of plasmids. </t>
   </si>
@@ -525,13 +526,196 @@
   </si>
   <si>
     <t>SiTag_in_pTwist_Chlor</t>
+  </si>
+  <si>
+    <t>OpenPichia MoClo - BCCM</t>
+  </si>
+  <si>
+    <t>pPTK001_P2_pAOX1</t>
+  </si>
+  <si>
+    <t>pPTK003_P4b_AOX1tt</t>
+  </si>
+  <si>
+    <t>pPTK004_P7_Stuffer</t>
+  </si>
+  <si>
+    <t>pPTK007_P4a_MYC-tag</t>
+  </si>
+  <si>
+    <t>pPTK008_P4a_HA-tag</t>
+  </si>
+  <si>
+    <t>pPTK010_P4a_HIS-tag</t>
+  </si>
+  <si>
+    <t>pPTK011_P7_ppARS1</t>
+  </si>
+  <si>
+    <t>pPTK016_P3a_ScMF</t>
+  </si>
+  <si>
+    <t>pPTK034_P2_pGAP</t>
+  </si>
+  <si>
+    <t>pPTK037_P3b_yEGFP</t>
+  </si>
+  <si>
+    <t>pPTK038_P4a_yEGFP</t>
+  </si>
+  <si>
+    <t>pPTK039_P7_HR1-Chr2</t>
+  </si>
+  <si>
+    <t>pPTK040_P7_HR1-Chr3</t>
+  </si>
+  <si>
+    <t>pPTK042_P6_BlastR</t>
+  </si>
+  <si>
+    <t>pPTK045_P7_HR1-Chr1</t>
+  </si>
+  <si>
+    <t>pPTK046_P7_HR1-Chr4</t>
+  </si>
+  <si>
+    <t>pPTK047_P4_AOX1tt</t>
+  </si>
+  <si>
+    <t>pPTK052_P4_DAS1tt</t>
+  </si>
+  <si>
+    <t>pPTK053_P4b_DAS1tt</t>
+  </si>
+  <si>
+    <t>pPTK054_P6_Stuffer</t>
+  </si>
+  <si>
+    <t>pPTK065_P6_HIS4</t>
+  </si>
+  <si>
+    <t>pPTK066_P6_Lox71-BlastR</t>
+  </si>
+  <si>
+    <t>pPTK068_P7_I-SceI_stuff</t>
+  </si>
+  <si>
+    <t>pPTK070_P1_ConLS</t>
+  </si>
+  <si>
+    <t>pPTK071_P1_ConL1</t>
+  </si>
+  <si>
+    <t>pPTK072_P1_ConLS'</t>
+  </si>
+  <si>
+    <t>pPTK073_P5_ConR1</t>
+  </si>
+  <si>
+    <t>pPTK074_P5_ConRE</t>
+  </si>
+  <si>
+    <t>pPTK075_P5_ConRE'</t>
+  </si>
+  <si>
+    <t>pPTK096_P3a_Ost1</t>
+  </si>
+  <si>
+    <t>pPTK109_P2-4_sfGFP</t>
+  </si>
+  <si>
+    <t>pPTK110_P3a_Kar2</t>
+  </si>
+  <si>
+    <t>pPTK146_P3b_sfGFP</t>
+  </si>
+  <si>
+    <t>pPTK147_P4a_sfGFP</t>
+  </si>
+  <si>
+    <t>pPTK188_P1_ConL2</t>
+  </si>
+  <si>
+    <t>pPTK189_P1_ConL3</t>
+  </si>
+  <si>
+    <t>pPTK190_P1_ConL4</t>
+  </si>
+  <si>
+    <t>pPTK191_P1_ConL5</t>
+  </si>
+  <si>
+    <t>pPTK192_P5_ConR2</t>
+  </si>
+  <si>
+    <t>pPTK193_P5_ConR3</t>
+  </si>
+  <si>
+    <t>pPTK194_P5_ConR4</t>
+  </si>
+  <si>
+    <t>pPTK195_P5_ConR5</t>
+  </si>
+  <si>
+    <t>pPTK200_P6_HygR</t>
+  </si>
+  <si>
+    <t>pPTK201_P6_NourR</t>
+  </si>
+  <si>
+    <t>pPTK202_P6_KanR</t>
+  </si>
+  <si>
+    <t>pPTK203_P6_ZeoR</t>
+  </si>
+  <si>
+    <t>pPTK204_P6_Lox71-HygR-L</t>
+  </si>
+  <si>
+    <t>pPTK205_P6_Lox71-NourR-</t>
+  </si>
+  <si>
+    <t>pPTK206_P6_Lox71-KanR-L</t>
+  </si>
+  <si>
+    <t>pPTK207_P6_Lox71-ZeoR-L</t>
+  </si>
+  <si>
+    <t>pPTK213_P3a_ScMFnoEAEA</t>
+  </si>
+  <si>
+    <t>pPTK076</t>
+  </si>
+  <si>
+    <t>pPTK077</t>
+  </si>
+  <si>
+    <t>pPTK078</t>
+  </si>
+  <si>
+    <t>pPTK079</t>
+  </si>
+  <si>
+    <t>pPTK080</t>
+  </si>
+  <si>
+    <t>pPTK196</t>
+  </si>
+  <si>
+    <t>pPTK197</t>
+  </si>
+  <si>
+    <t>pPTK198</t>
+  </si>
+  <si>
+    <t>pPTK199</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -550,6 +734,12 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1866,4 +2056,278 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0DDFAB60-9766-4B15-902C-DB155A00B5D2}">
+  <dimension ref="A1:M10"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>2</v>
+      </c>
+      <c r="D2">
+        <v>3</v>
+      </c>
+      <c r="E2">
+        <v>4</v>
+      </c>
+      <c r="F2">
+        <v>5</v>
+      </c>
+      <c r="G2">
+        <v>6</v>
+      </c>
+      <c r="H2">
+        <v>7</v>
+      </c>
+      <c r="I2">
+        <v>8</v>
+      </c>
+      <c r="J2">
+        <v>9</v>
+      </c>
+      <c r="K2">
+        <v>10</v>
+      </c>
+      <c r="L2">
+        <v>11</v>
+      </c>
+      <c r="M2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" t="s">
+        <v>163</v>
+      </c>
+      <c r="C3" t="s">
+        <v>164</v>
+      </c>
+      <c r="D3" t="s">
+        <v>165</v>
+      </c>
+      <c r="E3" t="s">
+        <v>166</v>
+      </c>
+      <c r="F3" t="s">
+        <v>167</v>
+      </c>
+      <c r="G3" t="s">
+        <v>168</v>
+      </c>
+      <c r="H3" t="s">
+        <v>169</v>
+      </c>
+      <c r="I3" t="s">
+        <v>170</v>
+      </c>
+      <c r="J3" t="s">
+        <v>171</v>
+      </c>
+      <c r="K3" t="s">
+        <v>172</v>
+      </c>
+      <c r="L3" t="s">
+        <v>173</v>
+      </c>
+      <c r="M3" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" t="s">
+        <v>187</v>
+      </c>
+      <c r="C4" t="s">
+        <v>175</v>
+      </c>
+      <c r="D4" t="s">
+        <v>176</v>
+      </c>
+      <c r="E4" t="s">
+        <v>177</v>
+      </c>
+      <c r="F4" t="s">
+        <v>178</v>
+      </c>
+      <c r="G4" t="s">
+        <v>179</v>
+      </c>
+      <c r="H4" t="s">
+        <v>180</v>
+      </c>
+      <c r="I4" t="s">
+        <v>181</v>
+      </c>
+      <c r="J4" t="s">
+        <v>182</v>
+      </c>
+      <c r="K4" t="s">
+        <v>183</v>
+      </c>
+      <c r="L4" t="s">
+        <v>184</v>
+      </c>
+      <c r="M4" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" t="s">
+        <v>186</v>
+      </c>
+      <c r="C5" t="s">
+        <v>188</v>
+      </c>
+      <c r="D5" t="s">
+        <v>189</v>
+      </c>
+      <c r="E5" t="s">
+        <v>190</v>
+      </c>
+      <c r="F5" t="s">
+        <v>191</v>
+      </c>
+      <c r="G5" t="s">
+        <v>214</v>
+      </c>
+      <c r="H5" t="s">
+        <v>215</v>
+      </c>
+      <c r="I5" t="s">
+        <v>216</v>
+      </c>
+      <c r="J5" t="s">
+        <v>217</v>
+      </c>
+      <c r="K5" t="s">
+        <v>218</v>
+      </c>
+      <c r="L5" t="s">
+        <v>192</v>
+      </c>
+      <c r="M5" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" t="s">
+        <v>194</v>
+      </c>
+      <c r="C6" t="s">
+        <v>195</v>
+      </c>
+      <c r="D6" t="s">
+        <v>196</v>
+      </c>
+      <c r="E6" t="s">
+        <v>197</v>
+      </c>
+      <c r="F6" t="s">
+        <v>198</v>
+      </c>
+      <c r="G6" t="s">
+        <v>199</v>
+      </c>
+      <c r="H6" t="s">
+        <v>200</v>
+      </c>
+      <c r="I6" t="s">
+        <v>201</v>
+      </c>
+      <c r="J6" t="s">
+        <v>202</v>
+      </c>
+      <c r="K6" t="s">
+        <v>203</v>
+      </c>
+      <c r="L6" t="s">
+        <v>204</v>
+      </c>
+      <c r="M6" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" t="s">
+        <v>220</v>
+      </c>
+      <c r="C7" t="s">
+        <v>221</v>
+      </c>
+      <c r="D7" t="s">
+        <v>222</v>
+      </c>
+      <c r="E7" t="s">
+        <v>205</v>
+      </c>
+      <c r="F7" t="s">
+        <v>206</v>
+      </c>
+      <c r="G7" t="s">
+        <v>207</v>
+      </c>
+      <c r="H7" t="s">
+        <v>208</v>
+      </c>
+      <c r="I7" t="s">
+        <v>209</v>
+      </c>
+      <c r="J7" t="s">
+        <v>210</v>
+      </c>
+      <c r="K7" t="s">
+        <v>211</v>
+      </c>
+      <c r="L7" t="s">
+        <v>212</v>
+      </c>
+      <c r="M7" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Added Human readable output for golden gate
</commit_message>
<xml_diff>
--- a/data/templates/TemPlates.xlsx
+++ b/data/templates/TemPlates.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\u5390772\Desktop\Code\PYEAST Local\data\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D22DF228-8826-4673-9617-DF0650F21D70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9033CD8F-3828-4042-95CF-34ACBFF817AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="16440" windowHeight="28320" firstSheet="1" activeTab="4" xr2:uid="{A88A2E90-7DAA-42AF-87DB-C66679F60F68}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="16440" windowHeight="28320" firstSheet="1" activeTab="1" xr2:uid="{A88A2E90-7DAA-42AF-87DB-C66679F60F68}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
-    <sheet name="TemPlate 1" sheetId="2" r:id="rId2"/>
-    <sheet name="YTK MoClo" sheetId="3" r:id="rId3"/>
-    <sheet name="YSD MoClo" sheetId="4" r:id="rId4"/>
-    <sheet name="Open Pichia" sheetId="5" r:id="rId5"/>
+    <sheet name="TemPlate_1" sheetId="2" r:id="rId2"/>
+    <sheet name="YTK_MoClo" sheetId="3" r:id="rId3"/>
+    <sheet name="YSD_MoClo" sheetId="4" r:id="rId4"/>
+    <sheet name="Open_Pichia" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>

</xml_diff>

<commit_message>
Updated bacth command and available templates for ANU availablity
</commit_message>
<xml_diff>
--- a/data/templates/TemPlates.xlsx
+++ b/data/templates/TemPlates.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\u5390772\Desktop\Code\PYEAST Local\data\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9033CD8F-3828-4042-95CF-34ACBFF817AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1764B6E-4497-419E-B5BC-11F9953F9CE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="16440" windowHeight="28320" firstSheet="1" activeTab="1" xr2:uid="{A88A2E90-7DAA-42AF-87DB-C66679F60F68}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="223">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="217">
   <si>
     <t xml:space="preserve">This is a database of templates useful for assembly of plasmids. </t>
   </si>
@@ -60,75 +60,30 @@
     <t>A</t>
   </si>
   <si>
-    <t>pESC-TRP</t>
-  </si>
-  <si>
-    <t>pVio_AmVHPO</t>
-  </si>
-  <si>
     <t>B</t>
   </si>
   <si>
-    <t>mCherry-pTwistAmp-Highcopy</t>
-  </si>
-  <si>
-    <t>Ty1Leu2int-AmpR</t>
-  </si>
-  <si>
     <t>C</t>
   </si>
   <si>
-    <t>pYES2-AmVHPO-ePTS1</t>
-  </si>
-  <si>
-    <t>pUC19</t>
-  </si>
-  <si>
-    <t>pUC19-POT1KO-His</t>
-  </si>
-  <si>
     <t>D</t>
   </si>
   <si>
     <t>BY4741</t>
   </si>
   <si>
-    <t>pYES2</t>
-  </si>
-  <si>
-    <t>pTw_Leu2MX_from_pRG205M</t>
-  </si>
-  <si>
     <t>E</t>
   </si>
   <si>
-    <t>pUC19-yEMRFP</t>
-  </si>
-  <si>
-    <t>pRS-AmVHPO-ePTS1</t>
-  </si>
-  <si>
     <t>F</t>
   </si>
   <si>
-    <t>s288c</t>
-  </si>
-  <si>
     <t>G</t>
   </si>
   <si>
-    <t>YeGFP-pTwistAmp-Highcopy</t>
-  </si>
-  <si>
     <t>H</t>
   </si>
   <si>
-    <t>pVio_Ura3_2u</t>
-  </si>
-  <si>
-    <t>pTw_His3MX</t>
-  </si>
-  <si>
     <t xml:space="preserve">YTK MoClo - Addgene </t>
   </si>
   <si>
@@ -709,6 +664,33 @@
   </si>
   <si>
     <t>pPTK199</t>
+  </si>
+  <si>
+    <t>pRG235</t>
+  </si>
+  <si>
+    <t>pRG203MX</t>
+  </si>
+  <si>
+    <t>pRG205MX</t>
+  </si>
+  <si>
+    <t>pRG206MX</t>
+  </si>
+  <si>
+    <t>Sitag</t>
+  </si>
+  <si>
+    <t>HyPer7</t>
+  </si>
+  <si>
+    <t>pSynOS_Alt4</t>
+  </si>
+  <si>
+    <t>SiTag_minilib1_4</t>
+  </si>
+  <si>
+    <t>SiTag_minilib1_3</t>
   </si>
 </sst>
 </file>
@@ -1187,87 +1169,69 @@
         <v>5</v>
       </c>
       <c r="B3" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C3" t="s">
-        <v>7</v>
+        <v>214</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>6</v>
+      </c>
+      <c r="B4" t="s">
+        <v>208</v>
       </c>
       <c r="C4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D4" t="s">
-        <v>10</v>
+        <v>213</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="B5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" t="s">
-        <v>13</v>
-      </c>
-      <c r="D5" t="s">
-        <v>14</v>
+        <v>209</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C6" t="s">
-        <v>17</v>
-      </c>
-      <c r="E6" t="s">
-        <v>18</v>
+        <v>210</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>20</v>
-      </c>
-      <c r="E7" t="s">
-        <v>21</v>
+        <v>211</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="B8" t="s">
-        <v>23</v>
-      </c>
-      <c r="E8" t="s">
-        <v>28</v>
+        <v>212</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="B9" t="s">
-        <v>25</v>
+        <v>216</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="B10" t="s">
-        <v>27</v>
+        <v>215</v>
       </c>
     </row>
   </sheetData>
@@ -1282,7 +1246,7 @@
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
@@ -1328,327 +1292,327 @@
         <v>5</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>33</v>
+        <v>18</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>34</v>
+        <v>19</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>36</v>
+        <v>21</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>37</v>
+        <v>22</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>39</v>
+        <v>24</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="L3" s="1" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="M3" s="1" t="s">
-        <v>42</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>43</v>
+        <v>28</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>44</v>
+        <v>29</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>46</v>
+        <v>31</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>47</v>
+        <v>32</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>48</v>
+        <v>33</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>52</v>
+        <v>37</v>
       </c>
       <c r="L4" s="1" t="s">
-        <v>53</v>
+        <v>38</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>54</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>55</v>
+        <v>40</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>56</v>
+        <v>41</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>57</v>
+        <v>42</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>58</v>
+        <v>43</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>59</v>
+        <v>44</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>62</v>
+        <v>47</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>63</v>
+        <v>48</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>64</v>
+        <v>49</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="M5" s="1" t="s">
-        <v>66</v>
+        <v>51</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>67</v>
+        <v>52</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>69</v>
+        <v>54</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>71</v>
+        <v>56</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>72</v>
+        <v>57</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>73</v>
+        <v>58</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>74</v>
+        <v>59</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>75</v>
+        <v>60</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>76</v>
+        <v>61</v>
       </c>
       <c r="L6" s="1" t="s">
-        <v>77</v>
+        <v>62</v>
       </c>
       <c r="M6" s="1" t="s">
-        <v>78</v>
+        <v>63</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>79</v>
+        <v>64</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>80</v>
+        <v>65</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>81</v>
+        <v>66</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>82</v>
+        <v>67</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>83</v>
+        <v>68</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>84</v>
+        <v>69</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>85</v>
+        <v>70</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>86</v>
+        <v>71</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>87</v>
+        <v>72</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>88</v>
+        <v>73</v>
       </c>
       <c r="L7" s="1" t="s">
-        <v>89</v>
+        <v>74</v>
       </c>
       <c r="M7" s="1" t="s">
-        <v>90</v>
+        <v>75</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>91</v>
+        <v>76</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>92</v>
+        <v>77</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>93</v>
+        <v>78</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>94</v>
+        <v>79</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>96</v>
+        <v>81</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>97</v>
+        <v>82</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>98</v>
+        <v>83</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>99</v>
+        <v>84</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>100</v>
+        <v>85</v>
       </c>
       <c r="L8" s="1" t="s">
-        <v>101</v>
+        <v>86</v>
       </c>
       <c r="M8" s="1" t="s">
-        <v>102</v>
+        <v>87</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>103</v>
+        <v>88</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>105</v>
+        <v>90</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>106</v>
+        <v>91</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>107</v>
+        <v>92</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>108</v>
+        <v>93</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>109</v>
+        <v>94</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>110</v>
+        <v>95</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>111</v>
+        <v>96</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>112</v>
+        <v>97</v>
       </c>
       <c r="L9" s="1" t="s">
-        <v>113</v>
+        <v>98</v>
       </c>
       <c r="M9" s="1" t="s">
-        <v>114</v>
+        <v>99</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>115</v>
+        <v>100</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>116</v>
+        <v>101</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>117</v>
+        <v>102</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>118</v>
+        <v>103</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>119</v>
+        <v>104</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>120</v>
+        <v>105</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>121</v>
+        <v>106</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>122</v>
+        <v>107</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>123</v>
+        <v>108</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>124</v>
+        <v>109</v>
       </c>
       <c r="L10" s="1" t="s">
-        <v>125</v>
+        <v>110</v>
       </c>
       <c r="M10" s="1" t="s">
-        <v>126</v>
+        <v>111</v>
       </c>
     </row>
   </sheetData>
@@ -1663,7 +1627,7 @@
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>30</v>
+        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
@@ -1709,144 +1673,144 @@
         <v>5</v>
       </c>
       <c r="B3" t="s">
-        <v>127</v>
+        <v>112</v>
       </c>
       <c r="C3" t="s">
-        <v>128</v>
+        <v>113</v>
       </c>
       <c r="D3" t="s">
-        <v>129</v>
+        <v>114</v>
       </c>
       <c r="E3" t="s">
-        <v>130</v>
+        <v>115</v>
       </c>
       <c r="F3" t="s">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="G3" t="s">
-        <v>132</v>
+        <v>117</v>
       </c>
       <c r="H3" t="s">
-        <v>133</v>
+        <v>118</v>
       </c>
       <c r="I3" t="s">
-        <v>134</v>
+        <v>119</v>
       </c>
       <c r="J3" t="s">
-        <v>135</v>
+        <v>120</v>
       </c>
       <c r="K3" t="s">
-        <v>136</v>
+        <v>121</v>
       </c>
       <c r="L3" t="s">
-        <v>137</v>
+        <v>122</v>
       </c>
       <c r="M3" t="s">
-        <v>138</v>
+        <v>123</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>139</v>
+        <v>124</v>
       </c>
       <c r="C4" t="s">
-        <v>140</v>
+        <v>125</v>
       </c>
       <c r="D4" t="s">
-        <v>141</v>
+        <v>126</v>
       </c>
       <c r="E4" t="s">
-        <v>142</v>
+        <v>127</v>
       </c>
       <c r="F4" t="s">
-        <v>143</v>
+        <v>128</v>
       </c>
       <c r="G4" t="s">
-        <v>144</v>
+        <v>129</v>
       </c>
       <c r="H4" t="s">
-        <v>145</v>
+        <v>130</v>
       </c>
       <c r="I4" t="s">
-        <v>146</v>
+        <v>131</v>
       </c>
       <c r="J4" t="s">
-        <v>147</v>
+        <v>132</v>
       </c>
       <c r="K4" t="s">
-        <v>148</v>
+        <v>133</v>
       </c>
       <c r="L4" t="s">
-        <v>149</v>
+        <v>134</v>
       </c>
       <c r="M4" t="s">
-        <v>150</v>
+        <v>135</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="B5" t="s">
-        <v>151</v>
+        <v>136</v>
       </c>
       <c r="C5" t="s">
-        <v>152</v>
+        <v>137</v>
       </c>
       <c r="D5" t="s">
-        <v>153</v>
+        <v>138</v>
       </c>
       <c r="E5" t="s">
-        <v>154</v>
+        <v>139</v>
       </c>
       <c r="F5" t="s">
-        <v>155</v>
+        <v>140</v>
       </c>
       <c r="G5" t="s">
-        <v>156</v>
+        <v>141</v>
       </c>
       <c r="H5" t="s">
-        <v>157</v>
+        <v>142</v>
       </c>
       <c r="I5" t="s">
-        <v>158</v>
+        <v>143</v>
       </c>
       <c r="J5" t="s">
-        <v>159</v>
+        <v>144</v>
       </c>
       <c r="K5" t="s">
-        <v>160</v>
+        <v>145</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="B10" t="s">
-        <v>161</v>
+        <v>146</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
@@ -2065,7 +2029,7 @@
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>162</v>
+        <v>147</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
@@ -2111,219 +2075,219 @@
         <v>5</v>
       </c>
       <c r="B3" t="s">
-        <v>163</v>
+        <v>148</v>
       </c>
       <c r="C3" t="s">
-        <v>164</v>
+        <v>149</v>
       </c>
       <c r="D3" t="s">
-        <v>165</v>
+        <v>150</v>
       </c>
       <c r="E3" t="s">
-        <v>166</v>
+        <v>151</v>
       </c>
       <c r="F3" t="s">
-        <v>167</v>
+        <v>152</v>
       </c>
       <c r="G3" t="s">
-        <v>168</v>
+        <v>153</v>
       </c>
       <c r="H3" t="s">
-        <v>169</v>
+        <v>154</v>
       </c>
       <c r="I3" t="s">
-        <v>170</v>
+        <v>155</v>
       </c>
       <c r="J3" t="s">
-        <v>171</v>
+        <v>156</v>
       </c>
       <c r="K3" t="s">
-        <v>172</v>
+        <v>157</v>
       </c>
       <c r="L3" t="s">
-        <v>173</v>
+        <v>158</v>
       </c>
       <c r="M3" t="s">
-        <v>174</v>
+        <v>159</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>187</v>
+        <v>172</v>
       </c>
       <c r="C4" t="s">
-        <v>175</v>
+        <v>160</v>
       </c>
       <c r="D4" t="s">
-        <v>176</v>
+        <v>161</v>
       </c>
       <c r="E4" t="s">
-        <v>177</v>
+        <v>162</v>
       </c>
       <c r="F4" t="s">
-        <v>178</v>
+        <v>163</v>
       </c>
       <c r="G4" t="s">
-        <v>179</v>
+        <v>164</v>
       </c>
       <c r="H4" t="s">
-        <v>180</v>
+        <v>165</v>
       </c>
       <c r="I4" t="s">
-        <v>181</v>
+        <v>166</v>
       </c>
       <c r="J4" t="s">
-        <v>182</v>
+        <v>167</v>
       </c>
       <c r="K4" t="s">
-        <v>183</v>
+        <v>168</v>
       </c>
       <c r="L4" t="s">
-        <v>184</v>
+        <v>169</v>
       </c>
       <c r="M4" t="s">
-        <v>185</v>
+        <v>170</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="B5" t="s">
-        <v>186</v>
+        <v>171</v>
       </c>
       <c r="C5" t="s">
-        <v>188</v>
+        <v>173</v>
       </c>
       <c r="D5" t="s">
-        <v>189</v>
+        <v>174</v>
       </c>
       <c r="E5" t="s">
-        <v>190</v>
+        <v>175</v>
       </c>
       <c r="F5" t="s">
-        <v>191</v>
+        <v>176</v>
       </c>
       <c r="G5" t="s">
-        <v>214</v>
+        <v>199</v>
       </c>
       <c r="H5" t="s">
-        <v>215</v>
+        <v>200</v>
       </c>
       <c r="I5" t="s">
-        <v>216</v>
+        <v>201</v>
       </c>
       <c r="J5" t="s">
-        <v>217</v>
+        <v>202</v>
       </c>
       <c r="K5" t="s">
-        <v>218</v>
+        <v>203</v>
       </c>
       <c r="L5" t="s">
-        <v>192</v>
+        <v>177</v>
       </c>
       <c r="M5" t="s">
-        <v>193</v>
+        <v>178</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>194</v>
+        <v>179</v>
       </c>
       <c r="C6" t="s">
-        <v>195</v>
+        <v>180</v>
       </c>
       <c r="D6" t="s">
-        <v>196</v>
+        <v>181</v>
       </c>
       <c r="E6" t="s">
-        <v>197</v>
+        <v>182</v>
       </c>
       <c r="F6" t="s">
-        <v>198</v>
+        <v>183</v>
       </c>
       <c r="G6" t="s">
-        <v>199</v>
+        <v>184</v>
       </c>
       <c r="H6" t="s">
-        <v>200</v>
+        <v>185</v>
       </c>
       <c r="I6" t="s">
-        <v>201</v>
+        <v>186</v>
       </c>
       <c r="J6" t="s">
-        <v>202</v>
+        <v>187</v>
       </c>
       <c r="K6" t="s">
-        <v>203</v>
+        <v>188</v>
       </c>
       <c r="L6" t="s">
+        <v>189</v>
+      </c>
+      <c r="M6" t="s">
         <v>204</v>
-      </c>
-      <c r="M6" t="s">
-        <v>219</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>220</v>
+        <v>205</v>
       </c>
       <c r="C7" t="s">
-        <v>221</v>
+        <v>206</v>
       </c>
       <c r="D7" t="s">
-        <v>222</v>
+        <v>207</v>
       </c>
       <c r="E7" t="s">
-        <v>205</v>
+        <v>190</v>
       </c>
       <c r="F7" t="s">
-        <v>206</v>
+        <v>191</v>
       </c>
       <c r="G7" t="s">
-        <v>207</v>
+        <v>192</v>
       </c>
       <c r="H7" t="s">
-        <v>208</v>
+        <v>193</v>
       </c>
       <c r="I7" t="s">
-        <v>209</v>
+        <v>194</v>
       </c>
       <c r="J7" t="s">
-        <v>210</v>
+        <v>195</v>
       </c>
       <c r="K7" t="s">
-        <v>211</v>
+        <v>196</v>
       </c>
       <c r="L7" t="s">
-        <v>212</v>
+        <v>197</v>
       </c>
       <c r="M7" t="s">
-        <v>213</v>
+        <v>198</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Bug fixes for batch command. Should now handle very large batches correctly
</commit_message>
<xml_diff>
--- a/data/templates/TemPlates.xlsx
+++ b/data/templates/TemPlates.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\u5390772\Desktop\Code\PYEAST Local\data\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1764B6E-4497-419E-B5BC-11F9953F9CE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94C4A9A4-0FB7-49A5-86FB-012C16BABD0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="16440" windowHeight="28320" firstSheet="1" activeTab="1" xr2:uid="{A88A2E90-7DAA-42AF-87DB-C66679F60F68}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="217">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="217">
   <si>
     <t xml:space="preserve">This is a database of templates useful for assembly of plasmids. </t>
   </si>
@@ -1193,6 +1193,9 @@
       <c r="B5" t="s">
         <v>209</v>
       </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">

</xml_diff>

<commit_message>
Cleaned up some private sequences
</commit_message>
<xml_diff>
--- a/data/templates/TemPlates.xlsx
+++ b/data/templates/TemPlates.xlsx
@@ -8,16 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\u5390772\Desktop\Code\PYEAST Local\data\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3453FC95-C759-49EA-8523-1156D6F73720}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD30F295-6514-497C-9710-4B582EA384DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-27630" yWindow="315" windowWidth="16410" windowHeight="11295" firstSheet="1" activeTab="1" xr2:uid="{A88A2E90-7DAA-42AF-87DB-C66679F60F68}"/>
+    <workbookView xWindow="-28920" yWindow="-975" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="3" xr2:uid="{A88A2E90-7DAA-42AF-87DB-C66679F60F68}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
     <sheet name="TemPlate_1" sheetId="2" r:id="rId2"/>
     <sheet name="YTK_MoClo" sheetId="3" r:id="rId3"/>
-    <sheet name="YSD_MoClo" sheetId="4" r:id="rId4"/>
-    <sheet name="Open_Pichia" sheetId="5" r:id="rId5"/>
+    <sheet name="Open_Pichia" sheetId="5" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -40,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="218">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="182">
   <si>
     <t xml:space="preserve">This is a database of templates useful for assembly of plasmids. </t>
   </si>
@@ -84,9 +83,6 @@
     <t xml:space="preserve">YTK MoClo - Addgene </t>
   </si>
   <si>
-    <t>YSD - MoClo Addgene</t>
-  </si>
-  <si>
     <t>pYTK001</t>
   </si>
   <si>
@@ -373,111 +369,6 @@
   </si>
   <si>
     <t>pYTK096</t>
-  </si>
-  <si>
-    <t>pYSD001</t>
-  </si>
-  <si>
-    <t>pYSD002</t>
-  </si>
-  <si>
-    <t>pYSD003</t>
-  </si>
-  <si>
-    <t>pYSD004</t>
-  </si>
-  <si>
-    <t>pYSD005</t>
-  </si>
-  <si>
-    <t>pYSD006</t>
-  </si>
-  <si>
-    <t>pYSD007</t>
-  </si>
-  <si>
-    <t>pYSD008</t>
-  </si>
-  <si>
-    <t>pYSD009</t>
-  </si>
-  <si>
-    <t>pYSD021</t>
-  </si>
-  <si>
-    <t>pYSD022</t>
-  </si>
-  <si>
-    <t>pYSD023</t>
-  </si>
-  <si>
-    <t>pYSD024</t>
-  </si>
-  <si>
-    <t>pYSD041</t>
-  </si>
-  <si>
-    <t>pYSD042</t>
-  </si>
-  <si>
-    <t>pYSD043</t>
-  </si>
-  <si>
-    <t>pYSD044</t>
-  </si>
-  <si>
-    <t>pYSD061</t>
-  </si>
-  <si>
-    <t>pYSD063</t>
-  </si>
-  <si>
-    <t>pYSD080</t>
-  </si>
-  <si>
-    <t>pYSD081</t>
-  </si>
-  <si>
-    <t>pYSD082</t>
-  </si>
-  <si>
-    <t>pYSD083</t>
-  </si>
-  <si>
-    <t>pYSD084</t>
-  </si>
-  <si>
-    <t>pYSD085</t>
-  </si>
-  <si>
-    <t>pYSD099</t>
-  </si>
-  <si>
-    <t>pYSD100</t>
-  </si>
-  <si>
-    <t>pYSD101</t>
-  </si>
-  <si>
-    <t>pYSD113</t>
-  </si>
-  <si>
-    <t>pYSD140</t>
-  </si>
-  <si>
-    <t>pYSD141</t>
-  </si>
-  <si>
-    <t>pYSD153</t>
-  </si>
-  <si>
-    <t>pYSD300</t>
-  </si>
-  <si>
-    <t>pYSD313</t>
-  </si>
-  <si>
-    <t>SiTag_in_pTwist_Chlor</t>
   </si>
   <si>
     <t>OpenPichia MoClo - BCCM</t>
@@ -1172,10 +1063,10 @@
         <v>5</v>
       </c>
       <c r="B3" t="s">
-        <v>217</v>
+        <v>181</v>
       </c>
       <c r="C3" t="s">
-        <v>216</v>
+        <v>180</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
@@ -1183,10 +1074,10 @@
         <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>215</v>
+        <v>179</v>
       </c>
       <c r="C4" t="s">
-        <v>214</v>
+        <v>178</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
@@ -1194,10 +1085,10 @@
         <v>7</v>
       </c>
       <c r="B5" t="s">
-        <v>213</v>
+        <v>177</v>
       </c>
       <c r="C5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
@@ -1205,10 +1096,10 @@
         <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>212</v>
+        <v>176</v>
       </c>
       <c r="C6" t="s">
-        <v>211</v>
+        <v>175</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
@@ -1216,7 +1107,7 @@
         <v>9</v>
       </c>
       <c r="B7" t="s">
-        <v>210</v>
+        <v>174</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
@@ -1224,7 +1115,7 @@
         <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>209</v>
+        <v>173</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
@@ -1232,7 +1123,7 @@
         <v>11</v>
       </c>
       <c r="B9" t="s">
-        <v>208</v>
+        <v>172</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
@@ -1240,7 +1131,7 @@
         <v>12</v>
       </c>
       <c r="B10" t="s">
-        <v>207</v>
+        <v>171</v>
       </c>
     </row>
   </sheetData>
@@ -1301,40 +1192,40 @@
         <v>5</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="D3" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="E3" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="F3" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="G3" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="H3" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="I3" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="I3" s="1" t="s">
+      <c r="J3" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="J3" s="1" t="s">
+      <c r="K3" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="K3" s="1" t="s">
+      <c r="L3" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="L3" s="1" t="s">
+      <c r="M3" s="1" t="s">
         <v>25</v>
-      </c>
-      <c r="M3" s="1" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
@@ -1342,40 +1233,40 @@
         <v>6</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="D4" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="E4" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="F4" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="G4" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="H4" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="I4" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="I4" s="1" t="s">
+      <c r="J4" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="J4" s="1" t="s">
+      <c r="K4" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="K4" s="1" t="s">
+      <c r="L4" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="L4" s="1" t="s">
+      <c r="M4" s="1" t="s">
         <v>37</v>
-      </c>
-      <c r="M4" s="1" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
@@ -1383,40 +1274,40 @@
         <v>7</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="D5" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="E5" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="F5" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="G5" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="H5" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="H5" s="1" t="s">
+      <c r="I5" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="I5" s="1" t="s">
+      <c r="J5" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="J5" s="1" t="s">
+      <c r="K5" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="K5" s="1" t="s">
+      <c r="L5" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="L5" s="1" t="s">
+      <c r="M5" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="M5" s="1" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
@@ -1424,40 +1315,40 @@
         <v>8</v>
       </c>
       <c r="B6" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="D6" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="E6" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="F6" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="G6" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="H6" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="H6" s="1" t="s">
+      <c r="I6" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="I6" s="1" t="s">
+      <c r="J6" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="J6" s="1" t="s">
+      <c r="K6" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="K6" s="1" t="s">
+      <c r="L6" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="L6" s="1" t="s">
+      <c r="M6" s="1" t="s">
         <v>61</v>
-      </c>
-      <c r="M6" s="1" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
@@ -1465,40 +1356,40 @@
         <v>9</v>
       </c>
       <c r="B7" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="D7" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="E7" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="F7" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="G7" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="G7" s="1" t="s">
+      <c r="H7" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="H7" s="1" t="s">
+      <c r="I7" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="I7" s="1" t="s">
+      <c r="J7" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="J7" s="1" t="s">
+      <c r="K7" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="K7" s="1" t="s">
+      <c r="L7" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="L7" s="1" t="s">
+      <c r="M7" s="1" t="s">
         <v>73</v>
-      </c>
-      <c r="M7" s="1" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
@@ -1506,40 +1397,40 @@
         <v>10</v>
       </c>
       <c r="B8" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="C8" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="D8" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="E8" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="F8" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="F8" s="1" t="s">
+      <c r="G8" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="G8" s="1" t="s">
+      <c r="H8" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="H8" s="1" t="s">
+      <c r="I8" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="I8" s="1" t="s">
+      <c r="J8" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="J8" s="1" t="s">
+      <c r="K8" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="K8" s="1" t="s">
+      <c r="L8" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="L8" s="1" t="s">
+      <c r="M8" s="1" t="s">
         <v>85</v>
-      </c>
-      <c r="M8" s="1" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
@@ -1547,40 +1438,40 @@
         <v>11</v>
       </c>
       <c r="B9" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C9" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="D9" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="D9" s="1" t="s">
+      <c r="E9" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="F9" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="G9" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="G9" s="1" t="s">
+      <c r="H9" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="H9" s="1" t="s">
+      <c r="I9" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="I9" s="1" t="s">
+      <c r="J9" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="J9" s="1" t="s">
+      <c r="K9" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="K9" s="1" t="s">
+      <c r="L9" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="L9" s="1" t="s">
+      <c r="M9" s="1" t="s">
         <v>97</v>
-      </c>
-      <c r="M9" s="1" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
@@ -1588,40 +1479,40 @@
         <v>12</v>
       </c>
       <c r="B10" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="D10" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="E10" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="F10" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="G10" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="G10" s="1" t="s">
+      <c r="H10" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="H10" s="1" t="s">
+      <c r="I10" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="I10" s="1" t="s">
+      <c r="J10" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="J10" s="1" t="s">
+      <c r="K10" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="K10" s="1" t="s">
+      <c r="L10" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="L10" s="1" t="s">
+      <c r="M10" s="1" t="s">
         <v>109</v>
-      </c>
-      <c r="M10" s="1" t="s">
-        <v>110</v>
       </c>
     </row>
   </sheetData>
@@ -1630,415 +1521,13 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8007E387-4B4E-4288-9FC9-B528CD4F9483}">
-  <dimension ref="A1:M72"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="B2">
-        <v>1</v>
-      </c>
-      <c r="C2">
-        <v>2</v>
-      </c>
-      <c r="D2">
-        <v>3</v>
-      </c>
-      <c r="E2">
-        <v>4</v>
-      </c>
-      <c r="F2">
-        <v>5</v>
-      </c>
-      <c r="G2">
-        <v>6</v>
-      </c>
-      <c r="H2">
-        <v>7</v>
-      </c>
-      <c r="I2">
-        <v>8</v>
-      </c>
-      <c r="J2">
-        <v>9</v>
-      </c>
-      <c r="K2">
-        <v>10</v>
-      </c>
-      <c r="L2">
-        <v>11</v>
-      </c>
-      <c r="M2">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" t="s">
-        <v>111</v>
-      </c>
-      <c r="C3" t="s">
-        <v>112</v>
-      </c>
-      <c r="D3" t="s">
-        <v>113</v>
-      </c>
-      <c r="E3" t="s">
-        <v>114</v>
-      </c>
-      <c r="F3" t="s">
-        <v>115</v>
-      </c>
-      <c r="G3" t="s">
-        <v>116</v>
-      </c>
-      <c r="H3" t="s">
-        <v>117</v>
-      </c>
-      <c r="I3" t="s">
-        <v>118</v>
-      </c>
-      <c r="J3" t="s">
-        <v>119</v>
-      </c>
-      <c r="K3" t="s">
-        <v>120</v>
-      </c>
-      <c r="L3" t="s">
-        <v>121</v>
-      </c>
-      <c r="M3" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" t="s">
-        <v>123</v>
-      </c>
-      <c r="C4" t="s">
-        <v>124</v>
-      </c>
-      <c r="D4" t="s">
-        <v>125</v>
-      </c>
-      <c r="E4" t="s">
-        <v>126</v>
-      </c>
-      <c r="F4" t="s">
-        <v>127</v>
-      </c>
-      <c r="G4" t="s">
-        <v>128</v>
-      </c>
-      <c r="H4" t="s">
-        <v>129</v>
-      </c>
-      <c r="I4" t="s">
-        <v>130</v>
-      </c>
-      <c r="J4" t="s">
-        <v>131</v>
-      </c>
-      <c r="K4" t="s">
-        <v>132</v>
-      </c>
-      <c r="L4" t="s">
-        <v>133</v>
-      </c>
-      <c r="M4" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5" t="s">
-        <v>135</v>
-      </c>
-      <c r="C5" t="s">
-        <v>136</v>
-      </c>
-      <c r="D5" t="s">
-        <v>137</v>
-      </c>
-      <c r="E5" t="s">
-        <v>138</v>
-      </c>
-      <c r="F5" t="s">
-        <v>139</v>
-      </c>
-      <c r="G5" t="s">
-        <v>140</v>
-      </c>
-      <c r="H5" t="s">
-        <v>141</v>
-      </c>
-      <c r="I5" t="s">
-        <v>142</v>
-      </c>
-      <c r="J5" t="s">
-        <v>143</v>
-      </c>
-      <c r="K5" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>12</v>
-      </c>
-      <c r="B10" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="C13" s="1"/>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="C14" s="1"/>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="C15" s="1"/>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="C16" s="1"/>
-    </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="C17" s="1"/>
-    </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="C18" s="1"/>
-    </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="C19" s="1"/>
-    </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="C20" s="1"/>
-    </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B21" s="1"/>
-      <c r="C21" s="1"/>
-      <c r="F21" s="1"/>
-    </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B22" s="1"/>
-      <c r="C22" s="1"/>
-      <c r="F22" s="1"/>
-    </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B23" s="1"/>
-      <c r="C23" s="1"/>
-      <c r="F23" s="1"/>
-    </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B24" s="1"/>
-      <c r="C24" s="1"/>
-      <c r="F24" s="1"/>
-    </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B25" s="1"/>
-      <c r="C25" s="1"/>
-      <c r="F25" s="1"/>
-    </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B26" s="1"/>
-      <c r="C26" s="1"/>
-      <c r="F26" s="1"/>
-    </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B27" s="1"/>
-      <c r="C27" s="1"/>
-      <c r="F27" s="1"/>
-    </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B28" s="1"/>
-      <c r="C28" s="1"/>
-      <c r="F28" s="1"/>
-    </row>
-    <row r="29" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B29" s="1"/>
-      <c r="C29" s="1"/>
-      <c r="F29" s="1"/>
-    </row>
-    <row r="30" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B30" s="1"/>
-      <c r="C30" s="1"/>
-      <c r="F30" s="1"/>
-    </row>
-    <row r="31" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B31" s="1"/>
-      <c r="C31" s="1"/>
-      <c r="F31" s="1"/>
-    </row>
-    <row r="32" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B32" s="1"/>
-      <c r="C32" s="1"/>
-      <c r="F32" s="1"/>
-    </row>
-    <row r="33" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C33" s="1"/>
-    </row>
-    <row r="34" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C34" s="1"/>
-    </row>
-    <row r="35" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C35" s="1"/>
-    </row>
-    <row r="36" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C36" s="1"/>
-    </row>
-    <row r="37" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C37" s="1"/>
-    </row>
-    <row r="38" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C38" s="1"/>
-    </row>
-    <row r="39" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C39" s="1"/>
-    </row>
-    <row r="40" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C40" s="1"/>
-    </row>
-    <row r="41" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C41" s="1"/>
-    </row>
-    <row r="42" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C42" s="1"/>
-    </row>
-    <row r="43" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C43" s="1"/>
-    </row>
-    <row r="44" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C44" s="1"/>
-    </row>
-    <row r="45" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C45" s="1"/>
-    </row>
-    <row r="46" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C46" s="1"/>
-    </row>
-    <row r="47" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C47" s="1"/>
-    </row>
-    <row r="48" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C48" s="1"/>
-    </row>
-    <row r="49" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C49" s="1"/>
-    </row>
-    <row r="50" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C50" s="1"/>
-    </row>
-    <row r="51" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C51" s="1"/>
-    </row>
-    <row r="52" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C52" s="1"/>
-    </row>
-    <row r="53" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C53" s="1"/>
-    </row>
-    <row r="54" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C54" s="1"/>
-    </row>
-    <row r="55" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C55" s="1"/>
-    </row>
-    <row r="56" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C56" s="1"/>
-    </row>
-    <row r="57" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C57" s="1"/>
-    </row>
-    <row r="58" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C58" s="1"/>
-    </row>
-    <row r="59" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C59" s="1"/>
-    </row>
-    <row r="60" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C60" s="1"/>
-    </row>
-    <row r="61" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C61" s="1"/>
-    </row>
-    <row r="62" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C62" s="1"/>
-    </row>
-    <row r="63" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C63" s="1"/>
-    </row>
-    <row r="64" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C64" s="1"/>
-    </row>
-    <row r="65" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C65" s="1"/>
-    </row>
-    <row r="66" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C66" s="1"/>
-    </row>
-    <row r="67" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C67" s="1"/>
-    </row>
-    <row r="68" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C68" s="1"/>
-    </row>
-    <row r="69" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C69" s="1"/>
-    </row>
-    <row r="70" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C70" s="1"/>
-    </row>
-    <row r="71" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C71" s="1"/>
-    </row>
-    <row r="72" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C72" s="1"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0DDFAB60-9766-4B15-902C-DB155A00B5D2}">
   <dimension ref="A1:M10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>146</v>
+        <v>110</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
@@ -2084,40 +1573,40 @@
         <v>5</v>
       </c>
       <c r="B3" t="s">
-        <v>147</v>
+        <v>111</v>
       </c>
       <c r="C3" t="s">
-        <v>148</v>
+        <v>112</v>
       </c>
       <c r="D3" t="s">
-        <v>149</v>
+        <v>113</v>
       </c>
       <c r="E3" t="s">
-        <v>150</v>
+        <v>114</v>
       </c>
       <c r="F3" t="s">
-        <v>151</v>
+        <v>115</v>
       </c>
       <c r="G3" t="s">
-        <v>152</v>
+        <v>116</v>
       </c>
       <c r="H3" t="s">
-        <v>153</v>
+        <v>117</v>
       </c>
       <c r="I3" t="s">
-        <v>154</v>
+        <v>118</v>
       </c>
       <c r="J3" t="s">
-        <v>155</v>
+        <v>119</v>
       </c>
       <c r="K3" t="s">
-        <v>156</v>
+        <v>120</v>
       </c>
       <c r="L3" t="s">
-        <v>157</v>
+        <v>121</v>
       </c>
       <c r="M3" t="s">
-        <v>158</v>
+        <v>122</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
@@ -2125,40 +1614,40 @@
         <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>171</v>
+        <v>135</v>
       </c>
       <c r="C4" t="s">
-        <v>159</v>
+        <v>123</v>
       </c>
       <c r="D4" t="s">
-        <v>160</v>
+        <v>124</v>
       </c>
       <c r="E4" t="s">
-        <v>161</v>
+        <v>125</v>
       </c>
       <c r="F4" t="s">
-        <v>162</v>
+        <v>126</v>
       </c>
       <c r="G4" t="s">
-        <v>163</v>
+        <v>127</v>
       </c>
       <c r="H4" t="s">
-        <v>164</v>
+        <v>128</v>
       </c>
       <c r="I4" t="s">
-        <v>165</v>
+        <v>129</v>
       </c>
       <c r="J4" t="s">
-        <v>166</v>
+        <v>130</v>
       </c>
       <c r="K4" t="s">
-        <v>167</v>
+        <v>131</v>
       </c>
       <c r="L4" t="s">
-        <v>168</v>
+        <v>132</v>
       </c>
       <c r="M4" t="s">
-        <v>169</v>
+        <v>133</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
@@ -2166,40 +1655,40 @@
         <v>7</v>
       </c>
       <c r="B5" t="s">
-        <v>170</v>
+        <v>134</v>
       </c>
       <c r="C5" t="s">
-        <v>172</v>
+        <v>136</v>
       </c>
       <c r="D5" t="s">
-        <v>173</v>
+        <v>137</v>
       </c>
       <c r="E5" t="s">
-        <v>174</v>
+        <v>138</v>
       </c>
       <c r="F5" t="s">
-        <v>175</v>
+        <v>139</v>
       </c>
       <c r="G5" t="s">
-        <v>198</v>
+        <v>162</v>
       </c>
       <c r="H5" t="s">
-        <v>199</v>
+        <v>163</v>
       </c>
       <c r="I5" t="s">
-        <v>200</v>
+        <v>164</v>
       </c>
       <c r="J5" t="s">
-        <v>201</v>
+        <v>165</v>
       </c>
       <c r="K5" t="s">
-        <v>202</v>
+        <v>166</v>
       </c>
       <c r="L5" t="s">
-        <v>176</v>
+        <v>140</v>
       </c>
       <c r="M5" t="s">
-        <v>177</v>
+        <v>141</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
@@ -2207,40 +1696,40 @@
         <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>178</v>
+        <v>142</v>
       </c>
       <c r="C6" t="s">
-        <v>179</v>
+        <v>143</v>
       </c>
       <c r="D6" t="s">
-        <v>180</v>
+        <v>144</v>
       </c>
       <c r="E6" t="s">
-        <v>181</v>
+        <v>145</v>
       </c>
       <c r="F6" t="s">
-        <v>182</v>
+        <v>146</v>
       </c>
       <c r="G6" t="s">
-        <v>183</v>
+        <v>147</v>
       </c>
       <c r="H6" t="s">
-        <v>184</v>
+        <v>148</v>
       </c>
       <c r="I6" t="s">
-        <v>185</v>
+        <v>149</v>
       </c>
       <c r="J6" t="s">
-        <v>186</v>
+        <v>150</v>
       </c>
       <c r="K6" t="s">
-        <v>187</v>
+        <v>151</v>
       </c>
       <c r="L6" t="s">
-        <v>188</v>
+        <v>152</v>
       </c>
       <c r="M6" t="s">
-        <v>203</v>
+        <v>167</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
@@ -2248,40 +1737,40 @@
         <v>9</v>
       </c>
       <c r="B7" t="s">
-        <v>204</v>
+        <v>168</v>
       </c>
       <c r="C7" t="s">
-        <v>205</v>
+        <v>169</v>
       </c>
       <c r="D7" t="s">
-        <v>206</v>
+        <v>170</v>
       </c>
       <c r="E7" t="s">
-        <v>189</v>
+        <v>153</v>
       </c>
       <c r="F7" t="s">
-        <v>190</v>
+        <v>154</v>
       </c>
       <c r="G7" t="s">
-        <v>191</v>
+        <v>155</v>
       </c>
       <c r="H7" t="s">
-        <v>192</v>
+        <v>156</v>
       </c>
       <c r="I7" t="s">
-        <v>193</v>
+        <v>157</v>
       </c>
       <c r="J7" t="s">
-        <v>194</v>
+        <v>158</v>
       </c>
       <c r="K7" t="s">
-        <v>195</v>
+        <v>159</v>
       </c>
       <c r="L7" t="s">
-        <v>196</v>
+        <v>160</v>
       </c>
       <c r="M7" t="s">
-        <v>197</v>
+        <v>161</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Minor update, added wheel>=0.46.2 dependancy to patch valunerability idenficied by dependabot
</commit_message>
<xml_diff>
--- a/data/templates/TemPlates.xlsx
+++ b/data/templates/TemPlates.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\u5390772\Desktop\Code\PYEAST Local\data\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD30F295-6514-497C-9710-4B582EA384DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52F80E56-2FA8-42FC-9B02-2AF9CBFACE00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-975" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="3" xr2:uid="{A88A2E90-7DAA-42AF-87DB-C66679F60F68}"/>
+    <workbookView xWindow="-28920" yWindow="-975" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{A88A2E90-7DAA-42AF-87DB-C66679F60F68}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="181">
   <si>
     <t xml:space="preserve">This is a database of templates useful for assembly of plasmids. </t>
   </si>
@@ -552,9 +552,6 @@
   </si>
   <si>
     <t>pPTK199</t>
-  </si>
-  <si>
-    <t>SiTag_minilib1_4</t>
   </si>
   <si>
     <t>SiTag_minilib1_3</t>
@@ -1063,10 +1060,10 @@
         <v>5</v>
       </c>
       <c r="B3" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C3" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
@@ -1074,10 +1071,10 @@
         <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C4" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
@@ -1085,7 +1082,7 @@
         <v>7</v>
       </c>
       <c r="B5" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C5" t="s">
         <v>14</v>
@@ -1096,10 +1093,10 @@
         <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C6" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
@@ -1107,7 +1104,7 @@
         <v>9</v>
       </c>
       <c r="B7" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
@@ -1115,7 +1112,7 @@
         <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
@@ -1123,15 +1120,12 @@
         <v>11</v>
       </c>
       <c r="B9" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>12</v>
-      </c>
-      <c r="B10" t="s">
-        <v>171</v>
       </c>
     </row>
   </sheetData>

</xml_diff>